<commit_message>
Refresh RSP and sanction-list sample data
Regenerate mock RSP files and the sanction list to include the new
Rule 202 cross-direction test scenarios.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input-rsp/RSP_Inbound_Apr26.xlsx
+++ b/input-rsp/RSP_Inbound_Apr26.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DQ4"/>
+  <dimension ref="A1:DQ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1116,43 +1116,133 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>901IBApr26</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>40000</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>ATH160001</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>Piti</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>2020000000901</t>
+        </is>
+      </c>
+      <c r="CK4" t="inlineStr">
+        <is>
+          <t>Self-Employed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>902IBApr26</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>ATH160001</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>Somchai</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>2020000000902</t>
+        </is>
+      </c>
+      <c r="CK5" t="inlineStr">
+        <is>
+          <t>Self-Employed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>203Apr26</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="L6" t="n">
         <v>20000</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>ATH160001</t>
         </is>
       </c>
-      <c r="BH4" t="inlineStr">
+      <c r="BH6" t="inlineStr">
         <is>
           <t>Nok</t>
         </is>
       </c>
-      <c r="BI4" t="inlineStr">
+      <c r="BI6" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="BV4" t="inlineStr">
+      <c r="BV6" t="inlineStr">
         <is>
           <t>2030000000203</t>
         </is>
       </c>
-      <c r="CK4" t="inlineStr">
+      <c r="CK6" t="inlineStr">
         <is>
           <t>Domestic Helper</t>
         </is>

</xml_diff>